<commit_message>
update score calculation table
</commit_message>
<xml_diff>
--- a/data/score-table.xlsx
+++ b/data/score-table.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <fileVersion appName="Calc"/>
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="51">
   <si>
     <t xml:space="preserve">Score</t>
   </si>
@@ -55,133 +55,121 @@
     <t xml:space="preserve">02:00:00</t>
   </si>
   <si>
-    <t xml:space="preserve">00:27:30</t>
-  </si>
-  <si>
-    <t xml:space="preserve">01:46:00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">00:25:00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">01:44:00</t>
-  </si>
-  <si>
     <t xml:space="preserve">00:23:00</t>
   </si>
   <si>
-    <t xml:space="preserve">01:42:00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">00:21:00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">01:39:40</t>
-  </si>
-  <si>
-    <t xml:space="preserve">00:20:00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">01:37:20</t>
-  </si>
-  <si>
-    <t xml:space="preserve">00:19:00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">01:35:00</t>
+    <t xml:space="preserve">01:50:00</t>
   </si>
   <si>
     <t xml:space="preserve">00:18:00</t>
   </si>
   <si>
-    <t xml:space="preserve">01:32:30</t>
+    <t xml:space="preserve">01:40:00</t>
   </si>
   <si>
     <t xml:space="preserve">00:17:00</t>
   </si>
   <si>
-    <t xml:space="preserve">01:29:50</t>
+    <t xml:space="preserve">01:38:00</t>
   </si>
   <si>
     <t xml:space="preserve">00:16:00</t>
   </si>
   <si>
-    <t xml:space="preserve">01:27:00</t>
+    <t xml:space="preserve">01:34:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">00:15:30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">01:31:00</t>
   </si>
   <si>
     <t xml:space="preserve">00:15:00</t>
   </si>
   <si>
-    <t xml:space="preserve">01:24:00</t>
+    <t xml:space="preserve">01:27:50</t>
+  </si>
+  <si>
+    <t xml:space="preserve">00:14:30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">01:23:00</t>
   </si>
   <si>
     <t xml:space="preserve">00:14:00</t>
   </si>
   <si>
-    <t xml:space="preserve">01:20:50</t>
+    <t xml:space="preserve">01:19:00</t>
   </si>
   <si>
     <t xml:space="preserve">00:13:30</t>
   </si>
   <si>
-    <t xml:space="preserve">01:17:40</t>
+    <t xml:space="preserve">01:16:00</t>
   </si>
   <si>
     <t xml:space="preserve">00:13:00</t>
   </si>
   <si>
-    <t xml:space="preserve">01:14:10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">00:12:30</t>
-  </si>
-  <si>
-    <t xml:space="preserve">01:10:40</t>
+    <t xml:space="preserve">01:13:30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">00:12:40</t>
+  </si>
+  <si>
+    <t xml:space="preserve">01:11:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">00:12:20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">01:08:30</t>
   </si>
   <si>
     <t xml:space="preserve">00:12:00</t>
   </si>
   <si>
-    <t xml:space="preserve">01:07:10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">00:11:30</t>
-  </si>
-  <si>
-    <t xml:space="preserve">01:03:40</t>
+    <t xml:space="preserve">01:06:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">00:11:40</t>
+  </si>
+  <si>
+    <t xml:space="preserve">01:03:30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">00:11:20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">01:01:00</t>
   </si>
   <si>
     <t xml:space="preserve">00:11:00</t>
   </si>
   <si>
-    <t xml:space="preserve">01:00:00</t>
+    <t xml:space="preserve">00:58:00</t>
   </si>
   <si>
     <t xml:space="preserve">00:10:30</t>
   </si>
   <si>
-    <t xml:space="preserve">00:56:00</t>
+    <t xml:space="preserve">00:55:00</t>
   </si>
   <si>
     <t xml:space="preserve">00:10:00</t>
   </si>
   <si>
-    <t xml:space="preserve">00:53:00</t>
+    <t xml:space="preserve">00:52:00</t>
   </si>
   <si>
     <t xml:space="preserve">00:09:30</t>
   </si>
   <si>
-    <t xml:space="preserve">00:50:00</t>
+    <t xml:space="preserve">00:49:00</t>
   </si>
   <si>
     <t xml:space="preserve">00:09:00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">00:47:40</t>
-  </si>
-  <si>
-    <t xml:space="preserve">00:08:00</t>
   </si>
   <si>
     <t xml:space="preserve">00:46:00</t>
@@ -609,7 +597,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:I25"/>
-  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="2" style="1" width="15.71"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="2" width="15.71"/>
@@ -652,18 +640,12 @@
       <c r="B2" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="C2" s="15" t="n">
-        <v>0</v>
-      </c>
+      <c r="C2" s="15"/>
       <c r="D2" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="E2" s="17" t="n">
-        <v>0</v>
-      </c>
-      <c r="F2" s="18" t="n">
-        <v>0</v>
-      </c>
+      <c r="E2" s="17"/>
+      <c r="F2" s="18"/>
       <c r="G2" s="19"/>
       <c r="H2" s="20" t="n">
         <v>0</v>
@@ -677,21 +659,15 @@
       <c r="B3" s="14" t="n">
         <v>2.02</v>
       </c>
-      <c r="C3" s="15" t="n">
-        <v>2.34</v>
-      </c>
+      <c r="C3" s="15"/>
       <c r="D3" s="16" t="n">
         <v>0.34</v>
       </c>
       <c r="E3" s="17"/>
       <c r="F3" s="18"/>
-      <c r="G3" s="19" t="s">
-        <v>9</v>
-      </c>
+      <c r="G3" s="19"/>
       <c r="H3" s="20"/>
-      <c r="I3" s="19" t="s">
-        <v>10</v>
-      </c>
+      <c r="I3" s="19"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="13" t="n">
@@ -700,25 +676,15 @@
       <c r="B4" s="14" t="n">
         <v>2.13</v>
       </c>
-      <c r="C4" s="15" t="n">
-        <v>2.61</v>
-      </c>
+      <c r="C4" s="15"/>
       <c r="D4" s="16" t="n">
         <v>0.36</v>
       </c>
-      <c r="E4" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="F4" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="G4" s="19" t="s">
-        <v>11</v>
-      </c>
+      <c r="E4" s="17"/>
+      <c r="F4" s="18"/>
+      <c r="G4" s="19"/>
       <c r="H4" s="20"/>
-      <c r="I4" s="19" t="s">
-        <v>12</v>
-      </c>
+      <c r="I4" s="19"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="13" t="n">
@@ -728,23 +694,25 @@
         <v>2.27</v>
       </c>
       <c r="C5" s="15" t="n">
-        <v>2.98</v>
+        <v>0</v>
       </c>
       <c r="D5" s="16" t="n">
         <v>0.4</v>
       </c>
       <c r="E5" s="17" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F5" s="18" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G5" s="19" t="s">
-        <v>13</v>
-      </c>
-      <c r="H5" s="20"/>
+        <v>9</v>
+      </c>
+      <c r="H5" s="20" t="n">
+        <v>10</v>
+      </c>
       <c r="I5" s="19" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -755,23 +723,25 @@
         <v>2.43</v>
       </c>
       <c r="C6" s="15" t="n">
-        <v>3.37</v>
+        <v>1</v>
       </c>
       <c r="D6" s="16" t="n">
         <v>0.44</v>
       </c>
       <c r="E6" s="17" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F6" s="18" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G6" s="19" t="s">
-        <v>15</v>
-      </c>
-      <c r="H6" s="20"/>
+        <v>11</v>
+      </c>
+      <c r="H6" s="20" t="n">
+        <v>50</v>
+      </c>
       <c r="I6" s="19" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -782,7 +752,7 @@
         <v>2.59</v>
       </c>
       <c r="C7" s="15" t="n">
-        <v>3.79</v>
+        <v>2</v>
       </c>
       <c r="D7" s="16" t="n">
         <v>0.48</v>
@@ -794,11 +764,13 @@
         <v>4</v>
       </c>
       <c r="G7" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="H7" s="20"/>
+        <v>13</v>
+      </c>
+      <c r="H7" s="20" t="n">
+        <v>100</v>
+      </c>
       <c r="I7" s="19" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -809,23 +781,25 @@
         <v>2.78</v>
       </c>
       <c r="C8" s="15" t="n">
-        <v>4.24</v>
+        <v>3</v>
       </c>
       <c r="D8" s="16" t="n">
         <v>0.52</v>
       </c>
       <c r="E8" s="17" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F8" s="18" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G8" s="19" t="s">
-        <v>19</v>
-      </c>
-      <c r="H8" s="20"/>
+        <v>15</v>
+      </c>
+      <c r="H8" s="20" t="n">
+        <v>150</v>
+      </c>
       <c r="I8" s="19" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -836,19 +810,25 @@
         <v>2.97</v>
       </c>
       <c r="C9" s="15" t="n">
-        <v>4.72</v>
+        <v>3.5</v>
       </c>
       <c r="D9" s="16" t="n">
         <v>0.57</v>
       </c>
-      <c r="E9" s="17"/>
-      <c r="F9" s="18"/>
+      <c r="E9" s="17" t="n">
+        <v>8</v>
+      </c>
+      <c r="F9" s="18" t="n">
+        <v>8</v>
+      </c>
       <c r="G9" s="19" t="s">
-        <v>21</v>
-      </c>
-      <c r="H9" s="20"/>
+        <v>17</v>
+      </c>
+      <c r="H9" s="20" t="n">
+        <v>200</v>
+      </c>
       <c r="I9" s="19" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -859,19 +839,25 @@
         <v>3.18</v>
       </c>
       <c r="C10" s="15" t="n">
-        <v>5.24</v>
+        <v>4</v>
       </c>
       <c r="D10" s="16" t="n">
         <v>0.62</v>
       </c>
-      <c r="E10" s="17"/>
-      <c r="F10" s="18"/>
+      <c r="E10" s="17" t="n">
+        <v>9</v>
+      </c>
+      <c r="F10" s="18" t="n">
+        <v>9</v>
+      </c>
       <c r="G10" s="19" t="s">
-        <v>23</v>
-      </c>
-      <c r="H10" s="20"/>
+        <v>19</v>
+      </c>
+      <c r="H10" s="20" t="n">
+        <v>250</v>
+      </c>
       <c r="I10" s="19" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -882,7 +868,7 @@
         <v>3.4</v>
       </c>
       <c r="C11" s="15" t="n">
-        <v>5.8</v>
+        <v>4.2</v>
       </c>
       <c r="D11" s="16" t="n">
         <v>0.68</v>
@@ -894,11 +880,13 @@
         <v>10</v>
       </c>
       <c r="G11" s="19" t="s">
-        <v>25</v>
-      </c>
-      <c r="H11" s="20"/>
+        <v>21</v>
+      </c>
+      <c r="H11" s="20" t="n">
+        <v>300</v>
+      </c>
       <c r="I11" s="19" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -909,19 +897,25 @@
         <v>3.64</v>
       </c>
       <c r="C12" s="15" t="n">
-        <v>6.4</v>
+        <v>4.4</v>
       </c>
       <c r="D12" s="16" t="n">
         <v>0.74</v>
       </c>
-      <c r="E12" s="17"/>
-      <c r="F12" s="18"/>
+      <c r="E12" s="17" t="n">
+        <v>11</v>
+      </c>
+      <c r="F12" s="18" t="n">
+        <v>11</v>
+      </c>
       <c r="G12" s="19" t="s">
-        <v>27</v>
-      </c>
-      <c r="H12" s="20"/>
+        <v>23</v>
+      </c>
+      <c r="H12" s="20" t="n">
+        <v>330</v>
+      </c>
       <c r="I12" s="19" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -932,19 +926,25 @@
         <v>3.89</v>
       </c>
       <c r="C13" s="15" t="n">
-        <v>7.03</v>
+        <v>4.6</v>
       </c>
       <c r="D13" s="16" t="n">
         <v>0.8</v>
       </c>
-      <c r="E13" s="17"/>
-      <c r="F13" s="18"/>
+      <c r="E13" s="17" t="n">
+        <v>12</v>
+      </c>
+      <c r="F13" s="18" t="n">
+        <v>12</v>
+      </c>
       <c r="G13" s="19" t="s">
-        <v>29</v>
-      </c>
-      <c r="H13" s="20"/>
+        <v>25</v>
+      </c>
+      <c r="H13" s="20" t="n">
+        <v>360</v>
+      </c>
       <c r="I13" s="19" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -955,19 +955,25 @@
         <v>4.16</v>
       </c>
       <c r="C14" s="15" t="n">
-        <v>7.7</v>
+        <v>4.8</v>
       </c>
       <c r="D14" s="16" t="n">
         <v>0.87</v>
       </c>
-      <c r="E14" s="17"/>
-      <c r="F14" s="18"/>
+      <c r="E14" s="17" t="n">
+        <v>13</v>
+      </c>
+      <c r="F14" s="18" t="n">
+        <v>13</v>
+      </c>
       <c r="G14" s="19" t="s">
-        <v>31</v>
-      </c>
-      <c r="H14" s="20"/>
+        <v>27</v>
+      </c>
+      <c r="H14" s="20" t="n">
+        <v>390</v>
+      </c>
       <c r="I14" s="19" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -978,19 +984,25 @@
         <v>4.45</v>
       </c>
       <c r="C15" s="15" t="n">
-        <v>8.42</v>
+        <v>5</v>
       </c>
       <c r="D15" s="16" t="n">
         <v>0.94</v>
       </c>
-      <c r="E15" s="17"/>
-      <c r="F15" s="18"/>
+      <c r="E15" s="17" t="n">
+        <v>14</v>
+      </c>
+      <c r="F15" s="18" t="n">
+        <v>14</v>
+      </c>
       <c r="G15" s="19" t="s">
-        <v>33</v>
-      </c>
-      <c r="H15" s="20"/>
+        <v>29</v>
+      </c>
+      <c r="H15" s="20" t="n">
+        <v>420</v>
+      </c>
       <c r="I15" s="19" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1001,19 +1013,25 @@
         <v>4.74</v>
       </c>
       <c r="C16" s="15" t="n">
-        <v>9.16</v>
+        <v>5.5</v>
       </c>
       <c r="D16" s="16" t="n">
         <v>1.01</v>
       </c>
-      <c r="E16" s="17"/>
-      <c r="F16" s="18"/>
+      <c r="E16" s="17" t="n">
+        <v>15</v>
+      </c>
+      <c r="F16" s="18" t="n">
+        <v>15</v>
+      </c>
       <c r="G16" s="19" t="s">
-        <v>35</v>
-      </c>
-      <c r="H16" s="20"/>
+        <v>31</v>
+      </c>
+      <c r="H16" s="20" t="n">
+        <v>450</v>
+      </c>
       <c r="I16" s="19" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1024,23 +1042,25 @@
         <v>5.06</v>
       </c>
       <c r="C17" s="15" t="n">
-        <v>9.94</v>
+        <v>6</v>
       </c>
       <c r="D17" s="16" t="n">
         <v>1.09</v>
       </c>
       <c r="E17" s="17" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="F17" s="18" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="G17" s="19" t="s">
-        <v>37</v>
-      </c>
-      <c r="H17" s="20"/>
+        <v>33</v>
+      </c>
+      <c r="H17" s="20" t="n">
+        <v>480</v>
+      </c>
       <c r="I17" s="19" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1051,19 +1071,25 @@
         <v>5.38</v>
       </c>
       <c r="C18" s="15" t="n">
-        <v>10.74</v>
+        <v>6.5</v>
       </c>
       <c r="D18" s="16" t="n">
         <v>1.17</v>
       </c>
-      <c r="E18" s="17"/>
-      <c r="F18" s="18"/>
+      <c r="E18" s="17" t="n">
+        <v>18</v>
+      </c>
+      <c r="F18" s="18" t="n">
+        <v>18</v>
+      </c>
       <c r="G18" s="19" t="s">
-        <v>39</v>
-      </c>
-      <c r="H18" s="20"/>
+        <v>35</v>
+      </c>
+      <c r="H18" s="20" t="n">
+        <v>510</v>
+      </c>
       <c r="I18" s="19" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1074,19 +1100,25 @@
         <v>5.71</v>
       </c>
       <c r="C19" s="15" t="n">
-        <v>11.56</v>
+        <v>7</v>
       </c>
       <c r="D19" s="16" t="n">
         <v>1.25</v>
       </c>
-      <c r="E19" s="17"/>
-      <c r="F19" s="18"/>
+      <c r="E19" s="17" t="n">
+        <v>20</v>
+      </c>
+      <c r="F19" s="18" t="n">
+        <v>20</v>
+      </c>
       <c r="G19" s="19" t="s">
-        <v>41</v>
-      </c>
-      <c r="H19" s="20"/>
+        <v>37</v>
+      </c>
+      <c r="H19" s="20" t="n">
+        <v>540</v>
+      </c>
       <c r="I19" s="19" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1097,19 +1129,25 @@
         <v>6.03</v>
       </c>
       <c r="C20" s="15" t="n">
-        <v>12.39</v>
+        <v>7.5</v>
       </c>
       <c r="D20" s="16" t="n">
         <v>1.34</v>
       </c>
-      <c r="E20" s="17"/>
-      <c r="F20" s="18"/>
+      <c r="E20" s="17" t="n">
+        <v>22</v>
+      </c>
+      <c r="F20" s="18" t="n">
+        <v>22</v>
+      </c>
       <c r="G20" s="19" t="s">
-        <v>43</v>
-      </c>
-      <c r="H20" s="20"/>
+        <v>39</v>
+      </c>
+      <c r="H20" s="20" t="n">
+        <v>570</v>
+      </c>
       <c r="I20" s="19" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1120,19 +1158,25 @@
         <v>6.36</v>
       </c>
       <c r="C21" s="15" t="n">
-        <v>13.2</v>
+        <v>8</v>
       </c>
       <c r="D21" s="16" t="n">
         <v>1.42</v>
       </c>
-      <c r="E21" s="17"/>
-      <c r="F21" s="18"/>
+      <c r="E21" s="17" t="n">
+        <v>24</v>
+      </c>
+      <c r="F21" s="18" t="n">
+        <v>24</v>
+      </c>
       <c r="G21" s="19" t="s">
-        <v>45</v>
-      </c>
-      <c r="H21" s="20"/>
+        <v>41</v>
+      </c>
+      <c r="H21" s="20" t="n">
+        <v>600</v>
+      </c>
       <c r="I21" s="19" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1143,23 +1187,25 @@
         <v>6.67</v>
       </c>
       <c r="C22" s="15" t="n">
-        <v>13.99</v>
+        <v>8.5</v>
       </c>
       <c r="D22" s="16" t="n">
         <v>1.49</v>
       </c>
       <c r="E22" s="17" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F22" s="18" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G22" s="19" t="s">
-        <v>47</v>
-      </c>
-      <c r="H22" s="20"/>
+        <v>43</v>
+      </c>
+      <c r="H22" s="20" t="n">
+        <v>650</v>
+      </c>
       <c r="I22" s="19" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1170,7 +1216,7 @@
         <v>6.97</v>
       </c>
       <c r="C23" s="15" t="n">
-        <v>14.72</v>
+        <v>9</v>
       </c>
       <c r="D23" s="16" t="n">
         <v>1.57</v>
@@ -1182,11 +1228,13 @@
         <v>28</v>
       </c>
       <c r="G23" s="19" t="s">
-        <v>49</v>
-      </c>
-      <c r="H23" s="20"/>
+        <v>45</v>
+      </c>
+      <c r="H23" s="20" t="n">
+        <v>700</v>
+      </c>
       <c r="I23" s="19" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1197,7 +1245,7 @@
         <v>7.24</v>
       </c>
       <c r="C24" s="15" t="n">
-        <v>15.39</v>
+        <v>9.5</v>
       </c>
       <c r="D24" s="16" t="n">
         <v>1.63</v>
@@ -1209,11 +1257,13 @@
         <v>29</v>
       </c>
       <c r="G24" s="19" t="s">
-        <v>51</v>
-      </c>
-      <c r="H24" s="20"/>
+        <v>47</v>
+      </c>
+      <c r="H24" s="20" t="n">
+        <v>800</v>
+      </c>
       <c r="I24" s="19" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1224,7 +1274,7 @@
         <v>7.47</v>
       </c>
       <c r="C25" s="15" t="n">
-        <v>15.96</v>
+        <v>10</v>
       </c>
       <c r="D25" s="16" t="n">
         <v>1.69</v>
@@ -1236,13 +1286,13 @@
         <v>30</v>
       </c>
       <c r="G25" s="19" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="H25" s="20" t="n">
-        <v>1100</v>
+        <v>900</v>
       </c>
       <c r="I25" s="19" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
udpate rules for biathlon
</commit_message>
<xml_diff>
--- a/data/score-table.xlsx
+++ b/data/score-table.xlsx
@@ -49,127 +49,127 @@
     <t xml:space="preserve">EKIDEN</t>
   </si>
   <si>
-    <t xml:space="preserve">00:30:00</t>
+    <t xml:space="preserve">00:10:00</t>
   </si>
   <si>
     <t xml:space="preserve">02:00:00</t>
   </si>
   <si>
-    <t xml:space="preserve">00:23:00</t>
+    <t xml:space="preserve">00:09:30</t>
   </si>
   <si>
     <t xml:space="preserve">01:50:00</t>
   </si>
   <si>
-    <t xml:space="preserve">00:18:00</t>
+    <t xml:space="preserve">00:09:00</t>
   </si>
   <si>
     <t xml:space="preserve">01:40:00</t>
   </si>
   <si>
-    <t xml:space="preserve">00:17:00</t>
+    <t xml:space="preserve">00:08:40</t>
   </si>
   <si>
     <t xml:space="preserve">01:38:00</t>
   </si>
   <si>
-    <t xml:space="preserve">00:16:00</t>
+    <t xml:space="preserve">00:08:20</t>
   </si>
   <si>
     <t xml:space="preserve">01:34:00</t>
   </si>
   <si>
-    <t xml:space="preserve">00:15:30</t>
+    <t xml:space="preserve">00:08:00</t>
   </si>
   <si>
     <t xml:space="preserve">01:31:00</t>
   </si>
   <si>
-    <t xml:space="preserve">00:15:00</t>
+    <t xml:space="preserve">00:07:40</t>
   </si>
   <si>
     <t xml:space="preserve">01:27:50</t>
   </si>
   <si>
-    <t xml:space="preserve">00:14:30</t>
+    <t xml:space="preserve">00:07:20</t>
   </si>
   <si>
     <t xml:space="preserve">01:23:00</t>
   </si>
   <si>
-    <t xml:space="preserve">00:14:00</t>
+    <t xml:space="preserve">00:07:00</t>
   </si>
   <si>
     <t xml:space="preserve">01:19:00</t>
   </si>
   <si>
-    <t xml:space="preserve">00:13:30</t>
+    <t xml:space="preserve">00:06:45</t>
   </si>
   <si>
     <t xml:space="preserve">01:16:00</t>
   </si>
   <si>
-    <t xml:space="preserve">00:13:00</t>
+    <t xml:space="preserve">00:06:30</t>
   </si>
   <si>
     <t xml:space="preserve">01:13:30</t>
   </si>
   <si>
-    <t xml:space="preserve">00:12:40</t>
+    <t xml:space="preserve">00:06:15</t>
   </si>
   <si>
     <t xml:space="preserve">01:11:00</t>
   </si>
   <si>
-    <t xml:space="preserve">00:12:20</t>
+    <t xml:space="preserve">00:06:00</t>
   </si>
   <si>
     <t xml:space="preserve">01:08:30</t>
   </si>
   <si>
-    <t xml:space="preserve">00:12:00</t>
+    <t xml:space="preserve">00:05:45</t>
   </si>
   <si>
     <t xml:space="preserve">01:06:00</t>
   </si>
   <si>
-    <t xml:space="preserve">00:11:40</t>
+    <t xml:space="preserve">00:05:30</t>
   </si>
   <si>
     <t xml:space="preserve">01:03:30</t>
   </si>
   <si>
-    <t xml:space="preserve">00:11:20</t>
+    <t xml:space="preserve">00:05:15</t>
   </si>
   <si>
     <t xml:space="preserve">01:01:00</t>
   </si>
   <si>
-    <t xml:space="preserve">00:11:00</t>
+    <t xml:space="preserve">00:05:00</t>
   </si>
   <si>
     <t xml:space="preserve">00:58:00</t>
   </si>
   <si>
-    <t xml:space="preserve">00:10:30</t>
+    <t xml:space="preserve">00:04:40</t>
   </si>
   <si>
     <t xml:space="preserve">00:55:00</t>
   </si>
   <si>
-    <t xml:space="preserve">00:10:00</t>
+    <t xml:space="preserve">00:04:20</t>
   </si>
   <si>
     <t xml:space="preserve">00:52:00</t>
   </si>
   <si>
-    <t xml:space="preserve">00:09:30</t>
+    <t xml:space="preserve">00:04:00</t>
   </si>
   <si>
     <t xml:space="preserve">00:49:00</t>
   </si>
   <si>
-    <t xml:space="preserve">00:09:00</t>
+    <t xml:space="preserve">00:03:40</t>
   </si>
   <si>
     <t xml:space="preserve">00:46:00</t>

</xml_diff>